<commit_message>
revenu: mise à jour de l'année de référence
fixes #517

La question doit être posée pour 2025
</commit_message>
<xml_diff>
--- a/survey/references/OD_nationale_quebec_2025.xlsx
+++ b/survey/references/OD_nationale_quebec_2025.xlsx
@@ -2278,7 +2278,7 @@
     <t xml:space="preserve">household.income</t>
   </si>
   <si>
-    <t xml:space="preserve">Tranche de revenu avant impôts (brut) du ménage, en 2024?
+    <t xml:space="preserve">Tranche de revenu avant impôts (brut) du ménage, en 2025?
 __Facultatif__</t>
   </si>
   <si>
@@ -2291,7 +2291,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">What was your household's income range before taxes (gross income), in 2024?
+      <t xml:space="preserve">What was your household's income range before taxes (gross income), in 2025?
 </t>
     </r>
     <r>

</xml_diff>